<commit_message>
changed mfn format: added network as additional parameter for nodes/paths/connections
</commit_message>
<xml_diff>
--- a/tests/formats/mfn_excel/MFN_Roboter_only.xlsx
+++ b/tests/formats/mfn_excel/MFN_Roboter_only.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\en986\Documents\Projects\Alltours\generalized_agv_path_finding\tests\formats\mfn_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35FCD83-2710-4636-ACE3-67A36B02660B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632DA370-C5E5-4DB8-BB4F-AB01BCC94BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{B8DE84FF-B3E8-4D87-8A95-BDBF8C6662ED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{B8DE84FF-B3E8-4D87-8A95-BDBF8C6662ED}"/>
   </bookViews>
   <sheets>
     <sheet name="NetworkNodes" sheetId="3" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="63">
   <si>
     <t>N</t>
   </si>
@@ -219,6 +219,9 @@
   </si>
   <si>
     <t>avg_speed_mps</t>
+  </si>
+  <si>
+    <t>Connection2</t>
   </si>
 </sst>
 </file>
@@ -1152,7 +1155,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -1167,10 +1170,10 @@
         <v>49</v>
       </c>
       <c r="F3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" t="s">
         <v>56</v>
-      </c>
-      <c r="G3" t="s">
-        <v>57</v>
       </c>
       <c r="I3" t="s">
         <v>50</v>

</xml_diff>